<commit_message>
feat: allow Excel re-upload to update profile and reset password for existing users
</commit_message>
<xml_diff>
--- a/Student_Import_Template.xlsx
+++ b/Student_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6cddac052b6f52f/Desktop/School project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4A49506-5379-4578-9A12-77959AED588D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{F4A49506-5379-4578-9A12-77959AED588D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BC9D01A-B27A-43E8-B427-A6417C5F5C06}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{039F3818-55B2-4C6A-8416-797342778AC8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>serial_no</t>
   </si>
@@ -87,24 +87,12 @@
     <t>A</t>
   </si>
   <si>
-    <t>Ramesh Sharma</t>
-  </si>
-  <si>
-    <t>Sunita Sharma</t>
-  </si>
-  <si>
     <t>Priya Reddy</t>
   </si>
   <si>
     <t>priya.reddy</t>
   </si>
   <si>
-    <t>Suresh Reddy</t>
-  </si>
-  <si>
-    <t>Kavitha Reddy</t>
-  </si>
-  <si>
     <t>Class Representative</t>
   </si>
   <si>
@@ -115,12 +103,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>Vijay Kumar</t>
-  </si>
-  <si>
-    <t>Meena Kumar</t>
   </si>
 </sst>
 </file>
@@ -553,12 +535,6 @@
       <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
       <c r="J2">
         <v>9876543210</v>
       </c>
@@ -571,10 +547,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
@@ -588,17 +564,11 @@
       <c r="G3" t="s">
         <v>16</v>
       </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
-      </c>
       <c r="J3">
         <v>9123456780</v>
       </c>
       <c r="L3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -606,10 +576,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
@@ -621,13 +591,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="J4">
         <v>9988776655</v>

</xml_diff>